<commit_message>
correción de HU (#55)
</commit_message>
<xml_diff>
--- a/Requisitos 💻/Historias de Usuario Scrum.xlsx
+++ b/Requisitos 💻/Historias de Usuario Scrum.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Ingenieria en Software\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Proyecto PeerHive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D5E3486-55D5-4EE9-8CA5-B27CD5F4A18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA225A75-C6FC-45FA-B5B4-D3EAD2F0AB9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="99">
   <si>
     <t>ID</t>
   </si>
@@ -313,6 +313,15 @@
   </si>
   <si>
     <t>Debe mostrarse nombre, rol e imagen de perfil del usuario.</t>
+  </si>
+  <si>
+    <t>HU-023</t>
+  </si>
+  <si>
+    <t>Como usuario, quiero realizar videollamadas dentro de la misma plataforma, para comunicarme a tiempo real con mi asesor o aprendiz.</t>
+  </si>
+  <si>
+    <t>La opción de “Iniciar videollamada” solo aparece una vez que la solicitud de ayuda ha sido aceptada.</t>
   </si>
 </sst>
 </file>
@@ -362,7 +371,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -398,24 +407,106 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="40% - Énfasis6" xfId="1" builtinId="51"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -466,10 +557,10 @@
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -495,7 +586,9 @@
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -547,62 +640,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -617,8 +654,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2FF29CC3-8A99-4B16-92CC-A09D5222D0D2}" name="Tabla1" displayName="Tabla1" ref="A1:E23" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="A1:E23" xr:uid="{2FF29CC3-8A99-4B16-92CC-A09D5222D0D2}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2FF29CC3-8A99-4B16-92CC-A09D5222D0D2}" name="Tabla1" displayName="Tabla1" ref="A1:E24" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E24" xr:uid="{2FF29CC3-8A99-4B16-92CC-A09D5222D0D2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -626,11 +663,11 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F46C5DF5-F757-41BD-8FA4-A7B85158D104}" name="ID" dataDxfId="6" dataCellStyle="40% - Énfasis6"/>
-    <tableColumn id="2" xr3:uid="{7A93D221-7E59-499A-AD97-4F368BB8CD2F}" name="Historia de Usuario" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{649C7636-00D1-4738-87EA-822B17E304BD}" name="Criterios de Aceptación" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F46C5DF5-F757-41BD-8FA4-A7B85158D104}" name="ID" dataDxfId="4" dataCellStyle="40% - Énfasis6"/>
+    <tableColumn id="2" xr3:uid="{7A93D221-7E59-499A-AD97-4F368BB8CD2F}" name="Historia de Usuario" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{649C7636-00D1-4738-87EA-822B17E304BD}" name="Criterios de Aceptación" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{A5834B82-093A-4850-9F9F-7B1657983E56}" name="Prioridad" dataDxfId="1" dataCellStyle="40% - Énfasis6"/>
-    <tableColumn id="6" xr3:uid="{F166956F-2C20-4DD4-BCF7-8B64890D6996}" name="Módulo / Funcionalidad" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{F166956F-2C20-4DD4-BCF7-8B64890D6996}" name="Módulo / Funcionalidad" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -957,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="132.7109375" customWidth="1"/>
@@ -1319,7 +1356,7 @@
         <v>60</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>85</v>
@@ -1357,6 +1394,23 @@
       </c>
       <c r="E23" s="2" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correción de requisito de Videollamas
</commit_message>
<xml_diff>
--- a/Requisitos 💻/Historias de Usuario Scrum.xlsx
+++ b/Requisitos 💻/Historias de Usuario Scrum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Proyecto PeerHive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA225A75-C6FC-45FA-B5B4-D3EAD2F0AB9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E9A7E4-7303-49D4-B04F-107C2DBFEB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -318,10 +318,10 @@
     <t>HU-023</t>
   </si>
   <si>
-    <t>Como usuario, quiero realizar videollamadas dentro de la misma plataforma, para comunicarme a tiempo real con mi asesor o aprendiz.</t>
-  </si>
-  <si>
     <t>La opción de “Iniciar videollamada” solo aparece una vez que la solicitud de ayuda ha sido aceptada.</t>
+  </si>
+  <si>
+    <t>Como usuario, quiero realizar videollamadas dentro de la misma plataforma, mediante API de Zoom.</t>
   </si>
 </sst>
 </file>
@@ -1401,10 +1401,10 @@
         <v>96</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>65</v>

</xml_diff>